<commit_message>
Slice 2: test case model, Excel writer, raised Coverage range
</commit_message>
<xml_diff>
--- a/templates/QA Test Case Template.xlsx
+++ b/templates/QA Test Case Template.xlsx
@@ -1104,23 +1104,23 @@
         </is>
       </c>
       <c r="B2" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A2)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A2)</f>
         <v/>
       </c>
       <c r="C2" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A2,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A2,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D2" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A2,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A2,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E2" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A2,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A2,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F2" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A2,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A2,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G2" s="23">
@@ -1135,23 +1135,23 @@
         </is>
       </c>
       <c r="B3" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A3)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A3)</f>
         <v/>
       </c>
       <c r="C3" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A3,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A3,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D3" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A3,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A3,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E3" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A3,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A3,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F3" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A3,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A3,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G3" s="23">
@@ -1166,23 +1166,23 @@
         </is>
       </c>
       <c r="B4" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A4)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A4,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A4,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D4" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A4,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A4,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E4" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A4,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A4,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F4" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A4,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A4,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G4" s="23">
@@ -1197,23 +1197,23 @@
         </is>
       </c>
       <c r="B5" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A5)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A5,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A5,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D5" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A5,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A5,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E5" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A5,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A5,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F5" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A5,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A5,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G5" s="23">
@@ -1228,23 +1228,23 @@
         </is>
       </c>
       <c r="B6" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A6)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A6,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A6,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D6" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A6,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A6,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A6,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A6,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A6,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A6,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G6" s="23">
@@ -1259,23 +1259,23 @@
         </is>
       </c>
       <c r="B7" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A7)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A7)</f>
         <v/>
       </c>
       <c r="C7" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A7,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A7,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D7" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A7,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A7,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E7" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A7,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A7,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F7" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A7,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A7,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G7" s="23">
@@ -1290,23 +1290,23 @@
         </is>
       </c>
       <c r="B8" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A8)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A8)</f>
         <v/>
       </c>
       <c r="C8" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A8,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A8,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D8" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A8,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A8,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A8,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A8,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A8,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A8,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G8" s="23">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="B9" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A9)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A9)</f>
         <v/>
       </c>
       <c r="C9" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A9,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A9,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D9" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A9,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A9,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E9" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A9,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A9,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F9" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A9,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A9,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G9" s="23">
@@ -1352,23 +1352,23 @@
         </is>
       </c>
       <c r="B10" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A10)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A10)</f>
         <v/>
       </c>
       <c r="C10" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A10,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A10,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D10" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A10,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A10,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A10,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A10,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A10,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A10,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G10" s="23">
@@ -1383,23 +1383,23 @@
         </is>
       </c>
       <c r="B11" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A11)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A11)</f>
         <v/>
       </c>
       <c r="C11" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A11,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A11,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D11" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A11,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A11,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E11" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A11,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A11,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F11" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A11,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A11,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G11" s="23">
@@ -1414,23 +1414,23 @@
         </is>
       </c>
       <c r="B12" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A12)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A12)</f>
         <v/>
       </c>
       <c r="C12" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A12,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A12,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A12,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A12,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A12,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A12,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A12,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A12,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G12" s="23">
@@ -1445,23 +1445,23 @@
         </is>
       </c>
       <c r="B13" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A13)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A13)</f>
         <v/>
       </c>
       <c r="C13" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A13,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A13,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A13,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A13,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A13,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A13,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F13" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A13,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A13,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G13" s="23">
@@ -1476,23 +1476,23 @@
         </is>
       </c>
       <c r="B14" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A14)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A14)</f>
         <v/>
       </c>
       <c r="C14" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A14,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A14,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A14,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A14,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A14,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A14,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F14" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A14,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A14,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G14" s="23">
@@ -1507,23 +1507,23 @@
         </is>
       </c>
       <c r="B15" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A15)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A15)</f>
         <v/>
       </c>
       <c r="C15" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A15,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A15,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A15,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A15,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A15,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A15,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F15" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A15,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A15,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G15" s="23">
@@ -1538,23 +1538,23 @@
         </is>
       </c>
       <c r="B16" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A16)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A16)</f>
         <v/>
       </c>
       <c r="C16" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A16,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A16,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A16,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A16,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A16,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A16,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F16" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A16,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A16,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G16" s="23">
@@ -1569,23 +1569,23 @@
         </is>
       </c>
       <c r="B17" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A17)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A17)</f>
         <v/>
       </c>
       <c r="C17" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A17,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A17,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A17,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A17,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A17,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A17,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F17" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A17,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A17,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G17" s="23">
@@ -1600,23 +1600,23 @@
         </is>
       </c>
       <c r="B18" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A18)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A18)</f>
         <v/>
       </c>
       <c r="C18" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A18,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A18,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A18,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A18,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A18,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A18,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F18" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A18,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A18,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G18" s="23">
@@ -1631,23 +1631,23 @@
         </is>
       </c>
       <c r="B19" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A19)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A19)</f>
         <v/>
       </c>
       <c r="C19" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A19,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A19,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A19,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A19,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A19,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A19,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F19" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A19,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A19,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G19" s="23">
@@ -1662,23 +1662,23 @@
         </is>
       </c>
       <c r="B20" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A20)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A20)</f>
         <v/>
       </c>
       <c r="C20" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A20,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A20,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A20,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A20,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A20,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A20,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F20" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A20,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A20,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G20" s="23">
@@ -1693,23 +1693,23 @@
         </is>
       </c>
       <c r="B21" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A21)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A21)</f>
         <v/>
       </c>
       <c r="C21" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A21,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A21,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A21,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A21,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A21,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A21,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F21" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A21,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A21,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G21" s="23">
@@ -1724,23 +1724,23 @@
         </is>
       </c>
       <c r="B22" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A22)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A22)</f>
         <v/>
       </c>
       <c r="C22" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A22,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A22,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A22,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A22,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A22,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A22,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F22" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A22,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A22,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G22" s="23">
@@ -1755,23 +1755,23 @@
         </is>
       </c>
       <c r="B23" s="22">
-        <f>COUNTIF('Functional Testing'!$M$2:$M$349,A23)</f>
+        <f>COUNTIF('Functional Testing'!$M$2:$M$2000,A23)</f>
         <v/>
       </c>
       <c r="C23" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A23,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A23,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D23" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A23,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A23,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E23" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A23,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A23,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F23" s="22">
-        <f>COUNTIFS('Functional Testing'!$M$2:$M$349,$A23,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$M$2:$M$2000,$A23,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G23" s="23">
@@ -1862,23 +1862,23 @@
         </is>
       </c>
       <c r="B28" s="22">
-        <f>COUNTIF('Functional Testing'!$K$2:$K$349,A28)</f>
+        <f>COUNTIF('Functional Testing'!$K$2:$K$2000,A28)</f>
         <v/>
       </c>
       <c r="C28" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A28,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A28,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A28,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A28,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A28,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A28,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F28" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A28,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A28,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G28" s="23">
@@ -1893,23 +1893,23 @@
         </is>
       </c>
       <c r="B29" s="22">
-        <f>COUNTIF('Functional Testing'!$K$2:$K$349,A29)</f>
+        <f>COUNTIF('Functional Testing'!$K$2:$K$2000,A29)</f>
         <v/>
       </c>
       <c r="C29" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A29,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A29,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D29" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A29,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A29,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E29" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A29,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A29,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F29" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A29,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A29,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G29" s="23">
@@ -1924,23 +1924,23 @@
         </is>
       </c>
       <c r="B30" s="22">
-        <f>COUNTIF('Functional Testing'!$K$2:$K$349,A30)</f>
+        <f>COUNTIF('Functional Testing'!$K$2:$K$2000,A30)</f>
         <v/>
       </c>
       <c r="C30" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A30,'Functional Testing'!$L$2:$L$349,"Pass")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A30,'Functional Testing'!$L$2:$L$2000,"Pass")</f>
         <v/>
       </c>
       <c r="D30" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A30,'Functional Testing'!$L$2:$L$349,"Fail")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A30,'Functional Testing'!$L$2:$L$2000,"Fail")</f>
         <v/>
       </c>
       <c r="E30" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A30,'Functional Testing'!$L$2:$L$349,"Blocked")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A30,'Functional Testing'!$L$2:$L$2000,"Blocked")</f>
         <v/>
       </c>
       <c r="F30" s="22">
-        <f>COUNTIFS('Functional Testing'!$K$2:$K$349,$A30,'Functional Testing'!$L$2:$L$349,"Not Executed")</f>
+        <f>COUNTIFS('Functional Testing'!$K$2:$K$2000,$A30,'Functional Testing'!$L$2:$L$2000,"Not Executed")</f>
         <v/>
       </c>
       <c r="G30" s="23">

</xml_diff>